<commit_message>
Cyclopean workbook: before/after comparison sheet with differences
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/cyclopean_ar.xlsx
+++ b/cyclopean_ar.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="الملخص" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="الإزاحة 1 م من وجه الخرسانة" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="بديل - الإزاحة من حد النظافة" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="المقارنة" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="الإزاحة 1 م من وجه الخرسانة" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="بديل - الإزاحة من حد النظافة" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'الإزاحة 1 م من وجه الخرسانة'!$5:$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'بديل - الإزاحة من حد النظافة'!$5:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'الإزاحة 1 م من وجه الخرسانة'!$5:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'بديل - الإزاحة من حد النظافة'!$5:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00;-#,##0.00;&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -111,8 +113,20 @@
       <color rgb="00008000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -139,8 +153,13 @@
         <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -176,11 +195,55 @@
         <color rgb="001F3864"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -227,6 +290,14 @@
     <xf numFmtId="164" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -236,6 +307,55 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -245,32 +365,14 @@
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -652,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E28"/>
+  <dimension ref="B2:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -941,127 +1043,93 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>الحفر قبل – على مساحة النظافة</t>
-        </is>
-      </c>
-      <c r="C21" s="15">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!G12</f>
-        <v>706.6720000000222</v>
-      </c>
-      <c r="D21" s="15">
-        <f>'بديل - الإزاحة من حد النظافة'!G12</f>
-        <v>706.6720000000222</v>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>م³</t>
-        </is>
-      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>• المعتمد: إزاحة 1 م من وجه الخرسانة (العمود الأول)؛ العمود الثاني للمقارنة فقط.</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>الحفر بعد – على مساحة السيكلوبين</t>
-        </is>
-      </c>
-      <c r="C22" s="14">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!H12</f>
-        <v>1072.5360000000337</v>
-      </c>
-      <c r="D22" s="14">
-        <f>'بديل - الإزاحة من حد النظافة'!H12</f>
-        <v>1114.325000000035</v>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>م³</t>
-        </is>
-      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>• الخلايا الصفراء في المعطيات قابلة للتعديل وتُحدّث كل الجداول تلقائياً.</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>الحفر الزائد</t>
         </is>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="21">
         <f>'الإزاحة 1 م من وجه الخرسانة'!I12</f>
         <v>365.8640000000115</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="21">
         <f>'بديل - الإزاحة من حد النظافة'!I12</f>
         <v>407.65300000001287</v>
       </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="E23" s="22" t="inlineStr">
         <is>
           <t>م³</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>خرسانة السيكلوبين (دبش + خرسانة)</t>
         </is>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="21">
         <f>'الإزاحة 1 م من وجه الخرسانة'!J12</f>
         <v>184.92000000000002</v>
       </c>
-      <c r="D24" s="17">
+      <c r="D24" s="21">
         <f>'بديل - الإزاحة من حد النظافة'!J12</f>
         <v>192.125</v>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr">
         <is>
           <t>م³</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="16" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>الردم الزائد</t>
         </is>
       </c>
-      <c r="C25" s="17">
+      <c r="C25" s="21">
         <f>'الإزاحة 1 م من وجه الخرسانة'!K12</f>
         <v>302.7840000000115</v>
       </c>
-      <c r="D25" s="17">
+      <c r="D25" s="21">
         <f>'بديل - الإزاحة من حد النظافة'!K12</f>
         <v>337.3680000000128</v>
       </c>
-      <c r="E25" s="18" t="inlineStr">
+      <c r="E25" s="22" t="inlineStr">
         <is>
           <t>م³</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="19" t="inlineStr">
-        <is>
-          <t>• المعتمد: إزاحة 1 م من وجه الخرسانة (العمود الأول)؛ العمود الثاني للمقارنة فقط.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>• الخلايا الصفراء في المعطيات قابلة للتعديل وتُحدّث كل الجداول تلقائياً.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B21:E21"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B22:E22"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1076,36 +1144,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K20"/>
+  <dimension ref="B2:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="2" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="2" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>جدول تفصيلي – الإزاحة 1 م من وجه الخرسانة</t>
+          <t>جدول مقارنة: قبل (الحفر على مساحة النظافة) – بعد (الحفر على مساحة السيكلوبين)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>المعتمد: الإزاحة 1.0 م مقيسة من وجه الخرسانة (0.9 م من حد النظافة) – بدون إزاحة على الوجه الخارجي للجدار الاستنادي</t>
-        </is>
-      </c>
+          <t>الإزاحة 1 م من وجه الخرسانة – الحفر من 1120.9 إلى 1118.0 – السيكلوبين من 1118.0 إلى 1118.5 – الردم من 1118.5 إلى 1120.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="B4" s="23" t="n"/>
+      <c r="C4" s="24" t="n"/>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>المساحة (م²)</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="n"/>
+      <c r="F4" s="24" t="n"/>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>الحفر (م³)</t>
+        </is>
+      </c>
+      <c r="H4" s="24" t="n"/>
+      <c r="I4" s="24" t="n"/>
+      <c r="J4" s="24" t="n"/>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>السيكلوبين (م³)</t>
+        </is>
+      </c>
+      <c r="L4" s="23" t="inlineStr">
+        <is>
+          <t>الردم (م³)</t>
+        </is>
+      </c>
+      <c r="M4" s="24" t="n"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
@@ -1120,400 +1220,401 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>مساحة النظافة
-(م²)</t>
+          <t>قبل
+(النظافة)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>مساحة السيكلوبين
-(م²)</t>
+          <t>بعد
+(السيكلوبين)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>مساحة شريط الإزاحة
-(م²)</t>
+          <t>الفرق</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>الحفر قبل
-على مساحة النظافة
-(م³)</t>
+          <t>قبل</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>الحفر بعد
-على مساحة السيكلوبين
-(م³)</t>
+          <t>بعد</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>الحفر الزائد
-(م³)</t>
+          <t>الفرق
+(زيادة)</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>خرسانة السيكلوبين
-(م³)</t>
+          <t>نسبة
+الزيادة</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>الردم الزائد
-(م³)</t>
+          <t>الكمية</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>قبل</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>بعد
+(الفرق)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="20" t="inlineStr"/>
-      <c r="C6" s="20" t="inlineStr"/>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>من الرسم</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>من الرسم</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>سيكلوبين − نظافة</t>
-        </is>
-      </c>
-      <c r="G6" s="20" t="inlineStr">
-        <is>
-          <t>نظافة × عمق الحفر</t>
-        </is>
-      </c>
-      <c r="H6" s="20" t="inlineStr">
-        <is>
-          <t>سيكلوبين × عمق الحفر</t>
-        </is>
-      </c>
-      <c r="I6" s="20" t="inlineStr">
-        <is>
-          <t>بعد − قبل</t>
-        </is>
-      </c>
-      <c r="J6" s="20" t="inlineStr">
-        <is>
-          <t>سيكلوبين × السماكة</t>
-        </is>
-      </c>
-      <c r="K6" s="20" t="inlineStr">
-        <is>
-          <t>شريط × ارتفاع الردم</t>
-        </is>
+      <c r="B6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة الجدار الاستنادي – الجزء الشمالي والشرقي</t>
+        </is>
+      </c>
+      <c r="D6" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!D7</f>
+        <v>180.09</v>
+      </c>
+      <c r="E6" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!E7</f>
+        <v>254.0</v>
+      </c>
+      <c r="F6" s="25">
+        <f>E6-D6</f>
+        <v>73.91</v>
+      </c>
+      <c r="G6" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G7</f>
+        <v>522.2610000000163</v>
+      </c>
+      <c r="H6" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H7</f>
+        <v>736.6000000000231</v>
+      </c>
+      <c r="I6" s="25">
+        <f>H6-G6</f>
+        <v>214.33900000000676</v>
+      </c>
+      <c r="J6" s="26">
+        <f>I6/G6</f>
+        <v>0.4104059081570327</v>
+      </c>
+      <c r="K6" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J7</f>
+        <v>127.0</v>
+      </c>
+      <c r="L6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="28">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!K7</f>
+        <v>177.38400000000672</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>قاعدة الجدار الاستنادي – الجزء الشمالي والشرقي</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="n">
-        <v>180.09</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <v>254</v>
-      </c>
-      <c r="F7" s="22">
+      <c r="B7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>قاعدة الجدار الاستنادي – الجزء الجنوبي والمنحنى</t>
+        </is>
+      </c>
+      <c r="D7" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!D8</f>
+        <v>38.65</v>
+      </c>
+      <c r="E7" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!E8</f>
+        <v>58.35</v>
+      </c>
+      <c r="F7" s="29">
         <f>E7-D7</f>
-        <v>73.91</v>
-      </c>
-      <c r="G7" s="22">
-        <f>D7*'الملخص'!$C$11</f>
-        <v>522.2610000000163</v>
-      </c>
-      <c r="H7" s="22">
-        <f>E7*'الملخص'!$C$11</f>
-        <v>736.6000000000231</v>
-      </c>
-      <c r="I7" s="23">
+        <v>19.700000000000003</v>
+      </c>
+      <c r="G7" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G8</f>
+        <v>112.08500000000352</v>
+      </c>
+      <c r="H7" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H8</f>
+        <v>169.21500000000532</v>
+      </c>
+      <c r="I7" s="29">
         <f>H7-G7</f>
-        <v>214.33900000000676</v>
-      </c>
-      <c r="J7" s="23">
-        <f>E7*'الملخص'!$C$9</f>
-        <v>127.0</v>
-      </c>
-      <c r="K7" s="23">
-        <f>F7*'الملخص'!$C$12</f>
-        <v>177.38400000000672</v>
+        <v>57.1300000000018</v>
+      </c>
+      <c r="J7" s="30">
+        <f>I7/G7</f>
+        <v>0.5097024579560155</v>
+      </c>
+      <c r="K7" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J8</f>
+        <v>29.175</v>
+      </c>
+      <c r="L7" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="32">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!K8</f>
+        <v>47.2800000000018</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>قاعدة الجدار الاستنادي – الجزء الجنوبي والمنحنى</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="n">
-        <v>38.65</v>
-      </c>
-      <c r="E8" s="24" t="n">
-        <v>58.35</v>
+      <c r="B8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P1</t>
+        </is>
+      </c>
+      <c r="D8" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!D9</f>
+        <v>14.44</v>
+      </c>
+      <c r="E8" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!E9</f>
+        <v>28.33</v>
       </c>
       <c r="F8" s="25">
         <f>E8-D8</f>
-        <v>19.700000000000003</v>
-      </c>
-      <c r="G8" s="25">
-        <f>D8*'الملخص'!$C$11</f>
-        <v>112.08500000000352</v>
-      </c>
-      <c r="H8" s="25">
-        <f>E8*'الملخص'!$C$11</f>
-        <v>169.21500000000532</v>
-      </c>
-      <c r="I8" s="26">
+        <v>13.889999999999999</v>
+      </c>
+      <c r="G8" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G9</f>
+        <v>41.87600000000131</v>
+      </c>
+      <c r="H8" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H9</f>
+        <v>82.15700000000257</v>
+      </c>
+      <c r="I8" s="25">
         <f>H8-G8</f>
-        <v>57.1300000000018</v>
+        <v>40.28100000000126</v>
       </c>
       <c r="J8" s="26">
-        <f>E8*'الملخص'!$C$9</f>
-        <v>29.175</v>
-      </c>
-      <c r="K8" s="26">
-        <f>F8*'الملخص'!$C$12</f>
-        <v>47.2800000000018</v>
+        <f>I8/G8</f>
+        <v>0.9619113573407201</v>
+      </c>
+      <c r="K8" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J9</f>
+        <v>14.165</v>
+      </c>
+      <c r="L8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="28">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!K9</f>
+        <v>33.33600000000126</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>قاعدة منفصلة P1</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="n">
-        <v>14.44</v>
-      </c>
-      <c r="E9" s="21" t="n">
-        <v>28.33</v>
-      </c>
-      <c r="F9" s="22">
+      <c r="B9" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P2</t>
+        </is>
+      </c>
+      <c r="D9" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!D10</f>
+        <v>5.25</v>
+      </c>
+      <c r="E9" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!E10</f>
+        <v>16.29</v>
+      </c>
+      <c r="F9" s="29">
         <f>E9-D9</f>
-        <v>13.889999999999999</v>
-      </c>
-      <c r="G9" s="22">
-        <f>D9*'الملخص'!$C$11</f>
-        <v>41.87600000000131</v>
-      </c>
-      <c r="H9" s="22">
-        <f>E9*'الملخص'!$C$11</f>
-        <v>82.15700000000257</v>
-      </c>
-      <c r="I9" s="23">
+        <v>11.04</v>
+      </c>
+      <c r="G9" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G10</f>
+        <v>15.225000000000477</v>
+      </c>
+      <c r="H9" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H10</f>
+        <v>47.24100000000148</v>
+      </c>
+      <c r="I9" s="29">
         <f>H9-G9</f>
-        <v>40.28100000000126</v>
-      </c>
-      <c r="J9" s="23">
-        <f>E9*'الملخص'!$C$9</f>
-        <v>14.165</v>
-      </c>
-      <c r="K9" s="23">
-        <f>F9*'الملخص'!$C$12</f>
-        <v>33.33600000000126</v>
+        <v>32.016000000001</v>
+      </c>
+      <c r="J9" s="30">
+        <f>I9/G9</f>
+        <v>2.1028571428571428</v>
+      </c>
+      <c r="K9" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J10</f>
+        <v>8.145</v>
+      </c>
+      <c r="L9" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="32">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!K10</f>
+        <v>26.496000000001</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>قاعدة منفصلة P2</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="n">
+      <c r="B10" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P3</t>
+        </is>
+      </c>
+      <c r="D10" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!D11</f>
         <v>5.25</v>
       </c>
-      <c r="E10" s="24" t="n">
-        <v>16.29</v>
+      <c r="E10" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!E11</f>
+        <v>12.87</v>
       </c>
       <c r="F10" s="25">
         <f>E10-D10</f>
-        <v>11.04</v>
-      </c>
-      <c r="G10" s="25">
-        <f>D10*'الملخص'!$C$11</f>
+        <v>7.619999999999999</v>
+      </c>
+      <c r="G10" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G11</f>
         <v>15.225000000000477</v>
       </c>
-      <c r="H10" s="25">
-        <f>E10*'الملخص'!$C$11</f>
-        <v>47.24100000000148</v>
-      </c>
-      <c r="I10" s="26">
+      <c r="H10" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H11</f>
+        <v>37.323000000001166</v>
+      </c>
+      <c r="I10" s="25">
         <f>H10-G10</f>
-        <v>32.016000000001</v>
+        <v>22.098000000000688</v>
       </c>
       <c r="J10" s="26">
-        <f>E10*'الملخص'!$C$9</f>
-        <v>8.145</v>
-      </c>
-      <c r="K10" s="26">
-        <f>F10*'الملخص'!$C$12</f>
-        <v>26.496000000001</v>
+        <f>I10/G10</f>
+        <v>1.451428571428571</v>
+      </c>
+      <c r="K10" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J11</f>
+        <v>6.435</v>
+      </c>
+      <c r="L10" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="28">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!K11</f>
+        <v>18.28800000000069</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>قاعدة منفصلة P3</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="E11" s="21" t="n">
-        <v>12.87</v>
-      </c>
-      <c r="F11" s="22">
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C11" s="34" t="n"/>
+      <c r="D11" s="35">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!D12</f>
+        <v>243.68</v>
+      </c>
+      <c r="E11" s="35">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!E12</f>
+        <v>369.84000000000003</v>
+      </c>
+      <c r="F11" s="36">
         <f>E11-D11</f>
-        <v>7.619999999999999</v>
-      </c>
-      <c r="G11" s="22">
-        <f>D11*'الملخص'!$C$11</f>
-        <v>15.225000000000477</v>
-      </c>
-      <c r="H11" s="22">
-        <f>E11*'الملخص'!$C$11</f>
-        <v>37.323000000001166</v>
-      </c>
-      <c r="I11" s="23">
+        <v>126.16000000000003</v>
+      </c>
+      <c r="G11" s="35">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G12</f>
+        <v>706.6720000000222</v>
+      </c>
+      <c r="H11" s="35">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H12</f>
+        <v>1072.5360000000337</v>
+      </c>
+      <c r="I11" s="36">
         <f>H11-G11</f>
-        <v>22.098000000000688</v>
-      </c>
-      <c r="J11" s="23">
-        <f>E11*'الملخص'!$C$9</f>
-        <v>6.435</v>
-      </c>
-      <c r="K11" s="23">
-        <f>F11*'الملخص'!$C$12</f>
-        <v>18.28800000000069</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>المجموع</t>
-        </is>
-      </c>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="29">
-        <f>SUM(D7:D11)</f>
-        <v>243.68</v>
-      </c>
-      <c r="E12" s="29">
-        <f>SUM(E7:E11)</f>
-        <v>369.84000000000003</v>
-      </c>
-      <c r="F12" s="29">
-        <f>SUM(F7:F11)</f>
-        <v>126.16</v>
-      </c>
-      <c r="G12" s="29">
-        <f>SUM(G7:G11)</f>
-        <v>706.6720000000222</v>
-      </c>
-      <c r="H12" s="29">
-        <f>SUM(H7:H11)</f>
-        <v>1072.5360000000337</v>
-      </c>
-      <c r="I12" s="29">
-        <f>SUM(I7:I11)</f>
         <v>365.8640000000115</v>
       </c>
-      <c r="J12" s="29">
-        <f>SUM(J7:J11)</f>
+      <c r="J11" s="37">
+        <f>I11/G11</f>
+        <v>0.5177281680892974</v>
+      </c>
+      <c r="K11" s="35">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J12</f>
         <v>184.92000000000002</v>
       </c>
-      <c r="K12" s="29">
-        <f>SUM(K7:K11)</f>
+      <c r="L11" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="35">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!K12</f>
         <v>302.7840000000115</v>
       </c>
     </row>
+    <row r="13">
+      <c r="B13" s="39" t="inlineStr">
+        <is>
+          <t>ملاحظات:</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="B14" s="30" t="inlineStr">
-        <is>
-          <t>ملاحظات:</t>
+      <c r="B14" s="40" t="inlineStr">
+        <is>
+          <t>• قبل: حفر القواعد على مساحة النظافة فقط (بدون سيكلوبين) – لا يوجد ردم إضافي.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>• مساحات النظافة والسيكلوبين مقيسة من ملف syclopien.dxf (التهشير الرمادي على طبقة S-D-WATER PROOF، وهو مرسوم على حد النظافة).</t>
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>• بعد: الحفر على مساحة السيكلوبين (القواعد + 1 م من وجه الخرسانة، بدون إزاحة على الوجه الخارجي للجدار الاستنادي).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>• في أماكن تداخل إزاحات القواعد المتجاورة وُزّعت المساحة المشتركة على أقرب قاعدة حتى لا تُحسب مرتين.</t>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>• الردم بعد = شريط الإزاحة حول القواعد فوق السيكلوبين (من 1118.5 إلى 1120.9)؛ لا يشمل الردم فوق القواعد نفسها.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>• الحفر الزائد = توسيع حفر القواعد بشريط الإزاحة من المنسوب العام حتى منسوب الحفر النهائي؛ لا يوجد حفر تحت هذا المنسوب.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>• الردم الزائد = شريط الإزاحة فوق السيكلوبين حتى المنسوب العام. لا يشمل الردم فوق القواعد نفسها لأنه موجود في الحالتين.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>• الجوانب محسوبة رأسية؛ أي ميول في جوانب الحفر تزيد الحفر والردم.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>• الخلايا الزرقاء قيم مقيسة من الرسم، والباقي معادلات مرتبطة بصفحة الملخص.</t>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>• الأرقام باللون الأحمر هي الفروقات الناتجة عن بند السيكلوبين؛ الأرقام الخضراء مرتبطة بصفحة التفصيل.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B14:K14"/>
-    <mergeCell ref="B17:K17"/>
-    <mergeCell ref="B18:K18"/>
-    <mergeCell ref="B16:K16"/>
-    <mergeCell ref="B15:K15"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B20:K20"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B19:K19"/>
-    <mergeCell ref="B12:C12"/>
+  <mergeCells count="12">
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B16:M16"/>
+    <mergeCell ref="B15:M15"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="B3:M3"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B14:M14"/>
+    <mergeCell ref="B17:M17"/>
+    <mergeCell ref="B13:M13"/>
+    <mergeCell ref="B4:C4"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1547,14 +1648,14 @@
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>جدول تفصيلي – بديل - الإزاحة من حد النظافة</t>
+          <t>جدول تفصيلي – الإزاحة 1 م من وجه الخرسانة</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>للمقارنة فقط: الإزاحة 1.0 م مقيسة من خط التهشير (حد النظافة) – بدون إزاحة على الوجه الخارجي للجدار الاستنادي</t>
+          <t>المعتمد: الإزاحة 1.0 م مقيسة من وجه الخرسانة (0.9 م من حد النظافة) – بدون إزاحة على الوجه الخارجي للجدار الاستنادي</t>
         </is>
       </c>
     </row>
@@ -1621,44 +1722,44 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="20" t="inlineStr"/>
-      <c r="C6" s="20" t="inlineStr"/>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr"/>
+      <c r="C6" s="41" t="inlineStr"/>
+      <c r="D6" s="41" t="inlineStr">
         <is>
           <t>من الرسم</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="41" t="inlineStr">
         <is>
           <t>من الرسم</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="41" t="inlineStr">
         <is>
           <t>سيكلوبين − نظافة</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="G6" s="41" t="inlineStr">
         <is>
           <t>نظافة × عمق الحفر</t>
         </is>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="H6" s="41" t="inlineStr">
         <is>
           <t>سيكلوبين × عمق الحفر</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr">
+      <c r="I6" s="41" t="inlineStr">
         <is>
           <t>بعد − قبل</t>
         </is>
       </c>
-      <c r="J6" s="20" t="inlineStr">
+      <c r="J6" s="41" t="inlineStr">
         <is>
           <t>سيكلوبين × السماكة</t>
         </is>
       </c>
-      <c r="K6" s="20" t="inlineStr">
+      <c r="K6" s="41" t="inlineStr">
         <is>
           <t>شريط × ارتفاع الردم</t>
         </is>
@@ -1673,35 +1774,35 @@
           <t>قاعدة الجدار الاستنادي – الجزء الشمالي والشرقي</t>
         </is>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="42" t="n">
         <v>180.09</v>
       </c>
-      <c r="E7" s="21" t="n">
-        <v>262.24</v>
-      </c>
-      <c r="F7" s="22">
+      <c r="E7" s="42" t="n">
+        <v>254</v>
+      </c>
+      <c r="F7" s="27">
         <f>E7-D7</f>
-        <v>82.15</v>
-      </c>
-      <c r="G7" s="22">
+        <v>73.91</v>
+      </c>
+      <c r="G7" s="27">
         <f>D7*'الملخص'!$C$11</f>
         <v>522.2610000000163</v>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="27">
         <f>E7*'الملخص'!$C$11</f>
-        <v>760.4960000000239</v>
-      </c>
-      <c r="I7" s="23">
+        <v>736.6000000000231</v>
+      </c>
+      <c r="I7" s="43">
         <f>H7-G7</f>
-        <v>238.23500000000752</v>
-      </c>
-      <c r="J7" s="23">
+        <v>214.33900000000676</v>
+      </c>
+      <c r="J7" s="43">
         <f>E7*'الملخص'!$C$9</f>
-        <v>131.12</v>
-      </c>
-      <c r="K7" s="23">
+        <v>127.0</v>
+      </c>
+      <c r="K7" s="43">
         <f>F7*'الملخص'!$C$12</f>
-        <v>197.16000000000747</v>
+        <v>177.38400000000672</v>
       </c>
     </row>
     <row r="8">
@@ -1713,35 +1814,35 @@
           <t>قاعدة الجدار الاستنادي – الجزء الجنوبي والمنحنى</t>
         </is>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="44" t="n">
         <v>38.65</v>
       </c>
-      <c r="E8" s="24" t="n">
-        <v>60.51</v>
-      </c>
-      <c r="F8" s="25">
+      <c r="E8" s="44" t="n">
+        <v>58.35</v>
+      </c>
+      <c r="F8" s="31">
         <f>E8-D8</f>
-        <v>21.86</v>
-      </c>
-      <c r="G8" s="25">
+        <v>19.700000000000003</v>
+      </c>
+      <c r="G8" s="31">
         <f>D8*'الملخص'!$C$11</f>
         <v>112.08500000000352</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="31">
         <f>E8*'الملخص'!$C$11</f>
-        <v>175.4790000000055</v>
-      </c>
-      <c r="I8" s="26">
+        <v>169.21500000000532</v>
+      </c>
+      <c r="I8" s="45">
         <f>H8-G8</f>
-        <v>63.39400000000198</v>
-      </c>
-      <c r="J8" s="26">
+        <v>57.1300000000018</v>
+      </c>
+      <c r="J8" s="45">
         <f>E8*'الملخص'!$C$9</f>
-        <v>30.255</v>
-      </c>
-      <c r="K8" s="26">
+        <v>29.175</v>
+      </c>
+      <c r="K8" s="45">
         <f>F8*'الملخص'!$C$12</f>
-        <v>52.46400000000199</v>
+        <v>47.2800000000018</v>
       </c>
     </row>
     <row r="9">
@@ -1753,35 +1854,35 @@
           <t>قاعدة منفصلة P1</t>
         </is>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="42" t="n">
         <v>14.44</v>
       </c>
-      <c r="E9" s="21" t="n">
-        <v>29.95</v>
-      </c>
-      <c r="F9" s="22">
+      <c r="E9" s="42" t="n">
+        <v>28.33</v>
+      </c>
+      <c r="F9" s="27">
         <f>E9-D9</f>
-        <v>15.51</v>
-      </c>
-      <c r="G9" s="22">
+        <v>13.889999999999999</v>
+      </c>
+      <c r="G9" s="27">
         <f>D9*'الملخص'!$C$11</f>
         <v>41.87600000000131</v>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="27">
         <f>E9*'الملخص'!$C$11</f>
-        <v>86.85500000000272</v>
-      </c>
-      <c r="I9" s="23">
+        <v>82.15700000000257</v>
+      </c>
+      <c r="I9" s="43">
         <f>H9-G9</f>
-        <v>44.979000000001406</v>
-      </c>
-      <c r="J9" s="23">
+        <v>40.28100000000126</v>
+      </c>
+      <c r="J9" s="43">
         <f>E9*'الملخص'!$C$9</f>
-        <v>14.975</v>
-      </c>
-      <c r="K9" s="23">
+        <v>14.165</v>
+      </c>
+      <c r="K9" s="43">
         <f>F9*'الملخص'!$C$12</f>
-        <v>37.22400000000141</v>
+        <v>33.33600000000126</v>
       </c>
     </row>
     <row r="10">
@@ -1793,35 +1894,35 @@
           <t>قاعدة منفصلة P2</t>
         </is>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="44" t="n">
         <v>5.25</v>
       </c>
-      <c r="E10" s="24" t="n">
-        <v>17.73</v>
-      </c>
-      <c r="F10" s="25">
+      <c r="E10" s="44" t="n">
+        <v>16.29</v>
+      </c>
+      <c r="F10" s="31">
         <f>E10-D10</f>
-        <v>12.48</v>
-      </c>
-      <c r="G10" s="25">
+        <v>11.04</v>
+      </c>
+      <c r="G10" s="31">
         <f>D10*'الملخص'!$C$11</f>
         <v>15.225000000000477</v>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="31">
         <f>E10*'الملخص'!$C$11</f>
-        <v>51.417000000001615</v>
-      </c>
-      <c r="I10" s="26">
+        <v>47.24100000000148</v>
+      </c>
+      <c r="I10" s="45">
         <f>H10-G10</f>
-        <v>36.19200000000114</v>
-      </c>
-      <c r="J10" s="26">
+        <v>32.016000000001</v>
+      </c>
+      <c r="J10" s="45">
         <f>E10*'الملخص'!$C$9</f>
-        <v>8.865</v>
-      </c>
-      <c r="K10" s="26">
+        <v>8.145</v>
+      </c>
+      <c r="K10" s="45">
         <f>F10*'الملخص'!$C$12</f>
-        <v>29.952000000001135</v>
+        <v>26.496000000001</v>
       </c>
     </row>
     <row r="11">
@@ -1833,121 +1934,572 @@
           <t>قاعدة منفصلة P3</t>
         </is>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="42" t="n">
         <v>5.25</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="42" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="F11" s="27">
+        <f>E11-D11</f>
+        <v>7.619999999999999</v>
+      </c>
+      <c r="G11" s="27">
+        <f>D11*'الملخص'!$C$11</f>
+        <v>15.225000000000477</v>
+      </c>
+      <c r="H11" s="27">
+        <f>E11*'الملخص'!$C$11</f>
+        <v>37.323000000001166</v>
+      </c>
+      <c r="I11" s="43">
+        <f>H11-G11</f>
+        <v>22.098000000000688</v>
+      </c>
+      <c r="J11" s="43">
+        <f>E11*'الملخص'!$C$9</f>
+        <v>6.435</v>
+      </c>
+      <c r="K11" s="43">
+        <f>F11*'الملخص'!$C$12</f>
+        <v>18.28800000000069</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="n"/>
+      <c r="D12" s="38">
+        <f>SUM(D7:D11)</f>
+        <v>243.68</v>
+      </c>
+      <c r="E12" s="38">
+        <f>SUM(E7:E11)</f>
+        <v>369.84000000000003</v>
+      </c>
+      <c r="F12" s="38">
+        <f>SUM(F7:F11)</f>
+        <v>126.16</v>
+      </c>
+      <c r="G12" s="38">
+        <f>SUM(G7:G11)</f>
+        <v>706.6720000000222</v>
+      </c>
+      <c r="H12" s="38">
+        <f>SUM(H7:H11)</f>
+        <v>1072.5360000000337</v>
+      </c>
+      <c r="I12" s="38">
+        <f>SUM(I7:I11)</f>
+        <v>365.8640000000115</v>
+      </c>
+      <c r="J12" s="38">
+        <f>SUM(J7:J11)</f>
+        <v>184.92000000000002</v>
+      </c>
+      <c r="K12" s="38">
+        <f>SUM(K7:K11)</f>
+        <v>302.7840000000115</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>ملاحظات:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>• مساحات النظافة والسيكلوبين مقيسة من ملف syclopien.dxf (التهشير الرمادي على طبقة S-D-WATER PROOF، وهو مرسوم على حد النظافة).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>• في أماكن تداخل إزاحات القواعد المتجاورة وُزّعت المساحة المشتركة على أقرب قاعدة حتى لا تُحسب مرتين.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>• الحفر الزائد = توسيع حفر القواعد بشريط الإزاحة من المنسوب العام حتى منسوب الحفر النهائي؛ لا يوجد حفر تحت هذا المنسوب.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="40" t="inlineStr">
+        <is>
+          <t>• الردم الزائد = شريط الإزاحة فوق السيكلوبين حتى المنسوب العام. لا يشمل الردم فوق القواعد نفسها لأنه موجود في الحالتين.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>• الجوانب محسوبة رأسية؛ أي ميول في جوانب الحفر تزيد الحفر والردم.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="40" t="inlineStr">
+        <is>
+          <t>• الخلايا الزرقاء قيم مقيسة من الرسم، والباقي معادلات مرتبطة بصفحة الملخص.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B14:K14"/>
+    <mergeCell ref="B17:K17"/>
+    <mergeCell ref="B18:K18"/>
+    <mergeCell ref="B16:K16"/>
+    <mergeCell ref="B15:K15"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B20:K20"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B19:K19"/>
+    <mergeCell ref="B12:C12"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:K20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="2" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>جدول تفصيلي – بديل - الإزاحة من حد النظافة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>للمقارنة فقط: الإزاحة 1.0 م مقيسة من خط التهشير (حد النظافة) – بدون إزاحة على الوجه الخارجي للجدار الاستنادي</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>القاعدة</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>مساحة النظافة
+(م²)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>مساحة السيكلوبين
+(م²)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>مساحة شريط الإزاحة
+(م²)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>الحفر قبل
+على مساحة النظافة
+(م³)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>الحفر بعد
+على مساحة السيكلوبين
+(م³)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>الحفر الزائد
+(م³)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>خرسانة السيكلوبين
+(م³)</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>الردم الزائد
+(م³)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="41" t="inlineStr"/>
+      <c r="C6" s="41" t="inlineStr"/>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>من الرسم</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>من الرسم</t>
+        </is>
+      </c>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>سيكلوبين − نظافة</t>
+        </is>
+      </c>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>نظافة × عمق الحفر</t>
+        </is>
+      </c>
+      <c r="H6" s="41" t="inlineStr">
+        <is>
+          <t>سيكلوبين × عمق الحفر</t>
+        </is>
+      </c>
+      <c r="I6" s="41" t="inlineStr">
+        <is>
+          <t>بعد − قبل</t>
+        </is>
+      </c>
+      <c r="J6" s="41" t="inlineStr">
+        <is>
+          <t>سيكلوبين × السماكة</t>
+        </is>
+      </c>
+      <c r="K6" s="41" t="inlineStr">
+        <is>
+          <t>شريط × ارتفاع الردم</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة الجدار الاستنادي – الجزء الشمالي والشرقي</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="n">
+        <v>180.09</v>
+      </c>
+      <c r="E7" s="42" t="n">
+        <v>262.24</v>
+      </c>
+      <c r="F7" s="27">
+        <f>E7-D7</f>
+        <v>82.15</v>
+      </c>
+      <c r="G7" s="27">
+        <f>D7*'الملخص'!$C$11</f>
+        <v>522.2610000000163</v>
+      </c>
+      <c r="H7" s="27">
+        <f>E7*'الملخص'!$C$11</f>
+        <v>760.4960000000239</v>
+      </c>
+      <c r="I7" s="43">
+        <f>H7-G7</f>
+        <v>238.23500000000752</v>
+      </c>
+      <c r="J7" s="43">
+        <f>E7*'الملخص'!$C$9</f>
+        <v>131.12</v>
+      </c>
+      <c r="K7" s="43">
+        <f>F7*'الملخص'!$C$12</f>
+        <v>197.16000000000747</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>قاعدة الجدار الاستنادي – الجزء الجنوبي والمنحنى</t>
+        </is>
+      </c>
+      <c r="D8" s="44" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="E8" s="44" t="n">
+        <v>60.51</v>
+      </c>
+      <c r="F8" s="31">
+        <f>E8-D8</f>
+        <v>21.86</v>
+      </c>
+      <c r="G8" s="31">
+        <f>D8*'الملخص'!$C$11</f>
+        <v>112.08500000000352</v>
+      </c>
+      <c r="H8" s="31">
+        <f>E8*'الملخص'!$C$11</f>
+        <v>175.4790000000055</v>
+      </c>
+      <c r="I8" s="45">
+        <f>H8-G8</f>
+        <v>63.39400000000198</v>
+      </c>
+      <c r="J8" s="45">
+        <f>E8*'الملخص'!$C$9</f>
+        <v>30.255</v>
+      </c>
+      <c r="K8" s="45">
+        <f>F8*'الملخص'!$C$12</f>
+        <v>52.46400000000199</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P1</t>
+        </is>
+      </c>
+      <c r="D9" s="42" t="n">
+        <v>14.44</v>
+      </c>
+      <c r="E9" s="42" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="F9" s="27">
+        <f>E9-D9</f>
+        <v>15.51</v>
+      </c>
+      <c r="G9" s="27">
+        <f>D9*'الملخص'!$C$11</f>
+        <v>41.87600000000131</v>
+      </c>
+      <c r="H9" s="27">
+        <f>E9*'الملخص'!$C$11</f>
+        <v>86.85500000000272</v>
+      </c>
+      <c r="I9" s="43">
+        <f>H9-G9</f>
+        <v>44.979000000001406</v>
+      </c>
+      <c r="J9" s="43">
+        <f>E9*'الملخص'!$C$9</f>
+        <v>14.975</v>
+      </c>
+      <c r="K9" s="43">
+        <f>F9*'الملخص'!$C$12</f>
+        <v>37.22400000000141</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P2</t>
+        </is>
+      </c>
+      <c r="D10" s="44" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="E10" s="44" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="F10" s="31">
+        <f>E10-D10</f>
+        <v>12.48</v>
+      </c>
+      <c r="G10" s="31">
+        <f>D10*'الملخص'!$C$11</f>
+        <v>15.225000000000477</v>
+      </c>
+      <c r="H10" s="31">
+        <f>E10*'الملخص'!$C$11</f>
+        <v>51.417000000001615</v>
+      </c>
+      <c r="I10" s="45">
+        <f>H10-G10</f>
+        <v>36.19200000000114</v>
+      </c>
+      <c r="J10" s="45">
+        <f>E10*'الملخص'!$C$9</f>
+        <v>8.865</v>
+      </c>
+      <c r="K10" s="45">
+        <f>F10*'الملخص'!$C$12</f>
+        <v>29.952000000001135</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P3</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="E11" s="42" t="n">
         <v>13.82</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="27">
         <f>E11-D11</f>
         <v>8.57</v>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="27">
         <f>D11*'الملخص'!$C$11</f>
         <v>15.225000000000477</v>
       </c>
-      <c r="H11" s="22">
+      <c r="H11" s="27">
         <f>E11*'الملخص'!$C$11</f>
         <v>40.07800000000126</v>
       </c>
-      <c r="I11" s="23">
+      <c r="I11" s="43">
         <f>H11-G11</f>
         <v>24.853000000000783</v>
       </c>
-      <c r="J11" s="23">
+      <c r="J11" s="43">
         <f>E11*'الملخص'!$C$9</f>
         <v>6.91</v>
       </c>
-      <c r="K11" s="23">
+      <c r="K11" s="43">
         <f>F11*'الملخص'!$C$12</f>
         <v>20.56800000000078</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="27" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>المجموع</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="29">
+      <c r="C12" s="34" t="n"/>
+      <c r="D12" s="38">
         <f>SUM(D7:D11)</f>
         <v>243.68</v>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="38">
         <f>SUM(E7:E11)</f>
         <v>384.25</v>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="38">
         <f>SUM(F7:F11)</f>
         <v>140.57</v>
       </c>
-      <c r="G12" s="29">
+      <c r="G12" s="38">
         <f>SUM(G7:G11)</f>
         <v>706.6720000000222</v>
       </c>
-      <c r="H12" s="29">
+      <c r="H12" s="38">
         <f>SUM(H7:H11)</f>
         <v>1114.325000000035</v>
       </c>
-      <c r="I12" s="29">
+      <c r="I12" s="38">
         <f>SUM(I7:I11)</f>
         <v>407.65300000001287</v>
       </c>
-      <c r="J12" s="29">
+      <c r="J12" s="38">
         <f>SUM(J7:J11)</f>
         <v>192.125</v>
       </c>
-      <c r="K12" s="29">
+      <c r="K12" s="38">
         <f>SUM(K7:K11)</f>
         <v>337.3680000000128</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="39" t="inlineStr">
         <is>
           <t>ملاحظات:</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t>• مساحات النظافة والسيكلوبين مقيسة من ملف syclopien.dxf (التهشير الرمادي على طبقة S-D-WATER PROOF، وهو مرسوم على حد النظافة).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B16" s="40" t="inlineStr">
         <is>
           <t>• في أماكن تداخل إزاحات القواعد المتجاورة وُزّعت المساحة المشتركة على أقرب قاعدة حتى لا تُحسب مرتين.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>• الحفر الزائد = توسيع حفر القواعد بشريط الإزاحة من المنسوب العام حتى منسوب الحفر النهائي؛ لا يوجد حفر تحت هذا المنسوب.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t>• الردم الزائد = شريط الإزاحة فوق السيكلوبين حتى المنسوب العام. لا يشمل الردم فوق القواعد نفسها لأنه موجود في الحالتين.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t>• الجوانب محسوبة رأسية؛ أي ميول في جوانب الحفر تزيد الحفر والردم.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t>• الخلايا الزرقاء قيم مقيسة من الرسم، والباقي معادلات مرتبطة بصفحة الملخص.</t>
         </is>

</xml_diff>

<commit_message>
Cyclopean: backfill = excavation - cyclopean - footing concrete - necks/walls, before vs after
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/cyclopean_ar.xlsx
+++ b/cyclopean_ar.xlsx
@@ -9,12 +9,13 @@
   <sheets>
     <sheet name="الملخص" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="المقارنة" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="الإزاحة 1 م من وجه الخرسانة" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="بديل - الإزاحة من حد النظافة" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="الردم" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="الإزاحة 1 م من وجه الخرسانة" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="بديل - الإزاحة من حد النظافة" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'الإزاحة 1 م من وجه الخرسانة'!$5:$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'بديل - الإزاحة من حد النظافة'!$5:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'الإزاحة 1 م من وجه الخرسانة'!$5:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'بديل - الإزاحة من حد النظافة'!$5:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -159,7 +160,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -195,55 +196,11 @@
         <color rgb="001F3864"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00A6A6A6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00A6A6A6"/>
-      </right>
-      <top style="thin">
-        <color rgb="00A6A6A6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00A6A6A6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00A6A6A6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00A6A6A6"/>
-      </right>
-      <top style="thin">
-        <color rgb="00A6A6A6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00A6A6A6"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -290,14 +247,6 @@
     <xf numFmtId="164" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -306,6 +255,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -317,61 +275,55 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -754,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E25"/>
+  <dimension ref="B2:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1043,93 +995,170 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>• المعتمد: إزاحة 1 م من وجه الخرسانة (العمود الأول)؛ العمود الثاني للمقارنة فقط.</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="n"/>
-      <c r="D21" s="17" t="n"/>
-      <c r="E21" s="18" t="n"/>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>الحفر قبل – على مساحة النظافة</t>
+        </is>
+      </c>
+      <c r="C21" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G12</f>
+        <v>706.6720000000222</v>
+      </c>
+      <c r="D21" s="15">
+        <f>'بديل - الإزاحة من حد النظافة'!G12</f>
+        <v>706.6720000000222</v>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>م³</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="B22" s="19" t="inlineStr">
-        <is>
-          <t>• الخلايا الصفراء في المعطيات قابلة للتعديل وتُحدّث كل الجداول تلقائياً.</t>
-        </is>
-      </c>
-      <c r="C22" s="17" t="n"/>
-      <c r="D22" s="17" t="n"/>
-      <c r="E22" s="18" t="n"/>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>الحفر بعد – على مساحة السيكلوبين</t>
+        </is>
+      </c>
+      <c r="C22" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H12</f>
+        <v>1072.5360000000337</v>
+      </c>
+      <c r="D22" s="14">
+        <f>'بديل - الإزاحة من حد النظافة'!H12</f>
+        <v>1114.325000000035</v>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>م³</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>الحفر الزائد</t>
         </is>
       </c>
-      <c r="C23" s="21">
+      <c r="C23" s="17">
         <f>'الإزاحة 1 م من وجه الخرسانة'!I12</f>
         <v>365.8640000000115</v>
       </c>
-      <c r="D23" s="21">
+      <c r="D23" s="17">
         <f>'بديل - الإزاحة من حد النظافة'!I12</f>
         <v>407.65300000001287</v>
       </c>
-      <c r="E23" s="22" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>م³</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>خرسانة السيكلوبين (دبش + خرسانة)</t>
         </is>
       </c>
-      <c r="C24" s="21">
+      <c r="C24" s="17">
         <f>'الإزاحة 1 م من وجه الخرسانة'!J12</f>
         <v>184.92000000000002</v>
       </c>
-      <c r="D24" s="21">
+      <c r="D24" s="17">
         <f>'بديل - الإزاحة من حد النظافة'!J12</f>
         <v>192.125</v>
       </c>
-      <c r="E24" s="22" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>م³</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>الردم الزائد</t>
-        </is>
-      </c>
-      <c r="C25" s="21">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!K12</f>
-        <v>302.7840000000115</v>
-      </c>
-      <c r="D25" s="21">
-        <f>'بديل - الإزاحة من حد النظافة'!K12</f>
-        <v>337.3680000000128</v>
-      </c>
-      <c r="E25" s="22" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>الردم قبل – حتى 1120.9</t>
+        </is>
+      </c>
+      <c r="C25" s="15">
+        <f>'الردم'!N20</f>
+        <v>486.1220000000152</v>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>م³</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>الردم بعد – حتى 1120.9</t>
+        </is>
+      </c>
+      <c r="C26" s="17">
+        <f>'الردم'!N11</f>
+        <v>686.3160000000266</v>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>م³</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>فرق الردم (زيادة)</t>
+        </is>
+      </c>
+      <c r="C27" s="20">
+        <f>C26-C25</f>
+        <v>200.19400000001144</v>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>م³</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>• المعتمد: إزاحة 1 م من وجه الخرسانة (العمود الأول)؛ العمود الثاني للمقارنة فقط.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>• الخلايا الصفراء في المعطيات قابلة للتعديل وتُحدّث كل الجداول تلقائياً.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="B30:E30"/>
     <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B29:E29"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B22:E22"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1144,7 +1173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:M17"/>
+  <dimension ref="B2:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1160,7 +1189,8 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="2" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="2" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
@@ -1178,34 +1208,35 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="B4" s="23" t="n"/>
-      <c r="C4" s="24" t="n"/>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="23" t="n"/>
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>المساحة (م²)</t>
         </is>
       </c>
-      <c r="E4" s="24" t="n"/>
-      <c r="F4" s="24" t="n"/>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="E4" s="23" t="n"/>
+      <c r="F4" s="23" t="n"/>
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>الحفر (م³)</t>
         </is>
       </c>
-      <c r="H4" s="24" t="n"/>
-      <c r="I4" s="24" t="n"/>
-      <c r="J4" s="24" t="n"/>
-      <c r="K4" s="23" t="inlineStr">
+      <c r="H4" s="23" t="n"/>
+      <c r="I4" s="23" t="n"/>
+      <c r="J4" s="23" t="n"/>
+      <c r="K4" s="22" t="inlineStr">
         <is>
           <t>السيكلوبين (م³)</t>
         </is>
       </c>
-      <c r="L4" s="23" t="inlineStr">
-        <is>
-          <t>الردم (م³)</t>
-        </is>
-      </c>
-      <c r="M4" s="24" t="n"/>
+      <c r="L4" s="22" t="inlineStr">
+        <is>
+          <t>الردم حتى 1120.9 (م³)</t>
+        </is>
+      </c>
+      <c r="M4" s="23" t="n"/>
+      <c r="N4" s="23" t="n"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
@@ -1269,8 +1300,12 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>بعد
-(الفرق)</t>
+          <t>بعد</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>الفرق</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1326,7 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!E7</f>
         <v>254.0</v>
       </c>
-      <c r="F6" s="25">
+      <c r="F6" s="24">
         <f>E6-D6</f>
         <v>73.91</v>
       </c>
@@ -1303,11 +1338,11 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!H7</f>
         <v>736.6000000000231</v>
       </c>
-      <c r="I6" s="25">
+      <c r="I6" s="24">
         <f>H6-G6</f>
         <v>214.33900000000676</v>
       </c>
-      <c r="J6" s="26">
+      <c r="J6" s="25">
         <f>I6/G6</f>
         <v>0.4104059081570327</v>
       </c>
@@ -1315,12 +1350,17 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!J7</f>
         <v>127.0</v>
       </c>
-      <c r="L6" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="28">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!K7</f>
-        <v>177.38400000000672</v>
+      <c r="L6" s="14">
+        <f>'الردم'!N15</f>
+        <v>356.08000000001107</v>
+      </c>
+      <c r="M6" s="14">
+        <f>'الردم'!N6</f>
+        <v>457.9440000000178</v>
+      </c>
+      <c r="N6" s="24">
+        <f>M6-L6</f>
+        <v>101.86400000000674</v>
       </c>
     </row>
     <row r="7">
@@ -1340,7 +1380,7 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!E8</f>
         <v>58.35</v>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="26">
         <f>E7-D7</f>
         <v>19.700000000000003</v>
       </c>
@@ -1352,11 +1392,11 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!H8</f>
         <v>169.21500000000532</v>
       </c>
-      <c r="I7" s="29">
+      <c r="I7" s="26">
         <f>H7-G7</f>
         <v>57.1300000000018</v>
       </c>
-      <c r="J7" s="30">
+      <c r="J7" s="27">
         <f>I7/G7</f>
         <v>0.5097024579560155</v>
       </c>
@@ -1364,12 +1404,17 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!J8</f>
         <v>29.175</v>
       </c>
-      <c r="L7" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="32">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!K8</f>
-        <v>47.2800000000018</v>
+      <c r="L7" s="15">
+        <f>'الردم'!N16</f>
+        <v>72.52500000000201</v>
+      </c>
+      <c r="M7" s="15">
+        <f>'الردم'!N7</f>
+        <v>104.64000000000378</v>
+      </c>
+      <c r="N7" s="26">
+        <f>M7-L7</f>
+        <v>32.11500000000177</v>
       </c>
     </row>
     <row r="8">
@@ -1389,7 +1434,7 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!E9</f>
         <v>28.33</v>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="24">
         <f>E8-D8</f>
         <v>13.889999999999999</v>
       </c>
@@ -1401,11 +1446,11 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!H9</f>
         <v>82.15700000000257</v>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="24">
         <f>H8-G8</f>
         <v>40.28100000000126</v>
       </c>
-      <c r="J8" s="26">
+      <c r="J8" s="25">
         <f>I8/G8</f>
         <v>0.9619113573407201</v>
       </c>
@@ -1413,12 +1458,17 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!J9</f>
         <v>14.165</v>
       </c>
-      <c r="L8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="28">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!K9</f>
-        <v>33.33600000000126</v>
+      <c r="L8" s="14">
+        <f>'الردم'!N17</f>
+        <v>32.97300000000123</v>
+      </c>
+      <c r="M8" s="14">
+        <f>'الردم'!N8</f>
+        <v>59.33400000000249</v>
+      </c>
+      <c r="N8" s="24">
+        <f>M8-L8</f>
+        <v>26.361000000001262</v>
       </c>
     </row>
     <row r="9">
@@ -1438,7 +1488,7 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!E10</f>
         <v>16.29</v>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="26">
         <f>E9-D9</f>
         <v>11.04</v>
       </c>
@@ -1450,11 +1500,11 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!H10</f>
         <v>47.24100000000148</v>
       </c>
-      <c r="I9" s="29">
+      <c r="I9" s="26">
         <f>H9-G9</f>
         <v>32.016000000001</v>
       </c>
-      <c r="J9" s="30">
+      <c r="J9" s="27">
         <f>I9/G9</f>
         <v>2.1028571428571428</v>
       </c>
@@ -1462,12 +1512,17 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!J10</f>
         <v>8.145</v>
       </c>
-      <c r="L9" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="32">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!K10</f>
-        <v>26.496000000001</v>
+      <c r="L9" s="15">
+        <f>'الردم'!N18</f>
+        <v>12.272000000000448</v>
+      </c>
+      <c r="M9" s="15">
+        <f>'الردم'!N9</f>
+        <v>36.30300000000145</v>
+      </c>
+      <c r="N9" s="26">
+        <f>M9-L9</f>
+        <v>24.031000000001</v>
       </c>
     </row>
     <row r="10">
@@ -1487,7 +1542,7 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!E11</f>
         <v>12.87</v>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="24">
         <f>E10-D10</f>
         <v>7.619999999999999</v>
       </c>
@@ -1499,11 +1554,11 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!H11</f>
         <v>37.323000000001166</v>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="24">
         <f>H10-G10</f>
         <v>22.098000000000688</v>
       </c>
-      <c r="J10" s="26">
+      <c r="J10" s="25">
         <f>I10/G10</f>
         <v>1.451428571428571</v>
       </c>
@@ -1511,91 +1566,101 @@
         <f>'الإزاحة 1 م من وجه الخرسانة'!J11</f>
         <v>6.435</v>
       </c>
-      <c r="L10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="28">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!K11</f>
-        <v>18.28800000000069</v>
+      <c r="L10" s="14">
+        <f>'الردم'!N19</f>
+        <v>12.272000000000448</v>
+      </c>
+      <c r="M10" s="14">
+        <f>'الردم'!N10</f>
+        <v>28.09500000000114</v>
+      </c>
+      <c r="N10" s="24">
+        <f>M10-L10</f>
+        <v>15.823000000000691</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="33" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>المجموع</t>
         </is>
       </c>
-      <c r="C11" s="34" t="n"/>
-      <c r="D11" s="35">
+      <c r="C11" s="29" t="n"/>
+      <c r="D11" s="30">
         <f>'الإزاحة 1 م من وجه الخرسانة'!D12</f>
         <v>243.68</v>
       </c>
-      <c r="E11" s="35">
+      <c r="E11" s="30">
         <f>'الإزاحة 1 م من وجه الخرسانة'!E12</f>
         <v>369.84000000000003</v>
       </c>
-      <c r="F11" s="36">
+      <c r="F11" s="31">
         <f>E11-D11</f>
         <v>126.16000000000003</v>
       </c>
-      <c r="G11" s="35">
+      <c r="G11" s="30">
         <f>'الإزاحة 1 م من وجه الخرسانة'!G12</f>
         <v>706.6720000000222</v>
       </c>
-      <c r="H11" s="35">
+      <c r="H11" s="30">
         <f>'الإزاحة 1 م من وجه الخرسانة'!H12</f>
         <v>1072.5360000000337</v>
       </c>
-      <c r="I11" s="36">
+      <c r="I11" s="31">
         <f>H11-G11</f>
         <v>365.8640000000115</v>
       </c>
-      <c r="J11" s="37">
+      <c r="J11" s="32">
         <f>I11/G11</f>
         <v>0.5177281680892974</v>
       </c>
-      <c r="K11" s="35">
+      <c r="K11" s="30">
         <f>'الإزاحة 1 م من وجه الخرسانة'!J12</f>
         <v>184.92000000000002</v>
       </c>
-      <c r="L11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="35">
-        <f>'الإزاحة 1 م من وجه الخرسانة'!K12</f>
-        <v>302.7840000000115</v>
+      <c r="L11" s="30">
+        <f>'الردم'!N20</f>
+        <v>486.1220000000152</v>
+      </c>
+      <c r="M11" s="30">
+        <f>'الردم'!N11</f>
+        <v>686.3160000000266</v>
+      </c>
+      <c r="N11" s="31">
+        <f>M11-L11</f>
+        <v>200.19400000001144</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="39" t="inlineStr">
+      <c r="B13" s="33" t="inlineStr">
         <is>
           <t>ملاحظات:</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="40" t="inlineStr">
-        <is>
-          <t>• قبل: حفر القواعد على مساحة النظافة فقط (بدون سيكلوبين) – لا يوجد ردم إضافي.</t>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>• قبل: حفر القواعد على مساحة النظافة فقط (بدون سيكلوبين)، والقواعد على منسوب 1118.0.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="40" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>• بعد: الحفر على مساحة السيكلوبين (القواعد + 1 م من وجه الخرسانة، بدون إزاحة على الوجه الخارجي للجدار الاستنادي).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t>• الردم بعد = شريط الإزاحة حول القواعد فوق السيكلوبين (من 1118.5 إلى 1120.9)؛ لا يشمل الردم فوق القواعد نفسها.</t>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>• الردم = الحفر − السيكلوبين − خرسانة القواعد − رقاب الأعمدة والجدران حتى 1120.9 (التفصيل في صفحة الردم).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="40" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>• الأرقام باللون الأحمر هي الفروقات الناتجة عن بند السيكلوبين؛ الأرقام الخضراء مرتبطة بصفحة التفصيل.</t>
         </is>
@@ -1603,17 +1668,17 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B16:M16"/>
-    <mergeCell ref="B15:M15"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="B3:M3"/>
+    <mergeCell ref="B16:N16"/>
+    <mergeCell ref="B14:N14"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="B14:M14"/>
-    <mergeCell ref="B17:M17"/>
-    <mergeCell ref="B13:M13"/>
+    <mergeCell ref="B17:N17"/>
+    <mergeCell ref="B13:N13"/>
+    <mergeCell ref="B15:N15"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="B2:N2"/>
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -1628,34 +1693,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K20"/>
+  <dimension ref="B2:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="2" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>جدول تفصيلي – الإزاحة 1 م من وجه الخرسانة</t>
+          <t>حساب الردم = الحفر − السيكلوبين − خرسانة القواعد − رقاب الأعمدة والجدران</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>المعتمد: الإزاحة 1.0 م مقيسة من وجه الخرسانة (0.9 م من حد النظافة) – بدون إزاحة على الوجه الخارجي للجدار الاستنادي</t>
+          <t>الردم حتى منسوب التسوية 1120.9 – الإزاحة 1 م من وجه الخرسانة</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>أولاً: بعد – القواعد على السيكلوبين (أسفل القاعدة 1118.5)، الحفر على مساحة السيكلوبين</t>
         </is>
       </c>
     </row>
@@ -1672,400 +1746,797 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>مساحة النظافة
-(م²)</t>
+          <t>سماكة القاعدة
+(م)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>مساحة السيكلوبين
-(م²)</t>
+          <t>منسوب أسفل
+القاعدة</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>مساحة شريط الإزاحة
-(م²)</t>
+          <t>منسوب سطح
+القاعدة</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>الحفر قبل
-على مساحة النظافة
+          <t>الحفر
 (م³)</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>الحفر بعد
-على مساحة السيكلوبين
+          <t>السيكلوبين
 (م³)</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>الحفر الزائد
+          <t>مساحة خرسانة
+القاعدة (م²)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>خرسانة القاعدة
 (م³)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>خرسانة السيكلوبين
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>مساحة الرقاب
+والجدران (م²)</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>ارتفاع الرقاب
+(م)</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>حجم الرقاب
+والجدران (م³)</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>الردم
 (م³)</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>الردم الزائد
+    </row>
+    <row r="6">
+      <c r="B6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة الجدار الاستنادي – الجزء الشمالي والشرقي</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E6" s="14">
+        <f>'الملخص'!$C$10</f>
+        <v>1118.5</v>
+      </c>
+      <c r="F6" s="35">
+        <f>E6+D6</f>
+        <v>1119.1</v>
+      </c>
+      <c r="G6" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H7</f>
+        <v>736.6000000000231</v>
+      </c>
+      <c r="H6" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J7</f>
+        <v>127.0</v>
+      </c>
+      <c r="I6" s="34" t="n">
+        <v>165.61</v>
+      </c>
+      <c r="J6" s="35">
+        <f>I6*D6</f>
+        <v>99.366</v>
+      </c>
+      <c r="K6" s="34" t="n">
+        <v>29.05</v>
+      </c>
+      <c r="L6" s="35">
+        <f>'الملخص'!$C$7-F6</f>
+        <v>1.800000000000182</v>
+      </c>
+      <c r="M6" s="35">
+        <f>K6*L6</f>
+        <v>52.290000000005286</v>
+      </c>
+      <c r="N6" s="36">
+        <f>G6-H6-J6-M6</f>
+        <v>457.9440000000178</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>قاعدة الجدار الاستنادي – الجزء الجنوبي والمنحنى</t>
+        </is>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E7" s="15">
+        <f>'الملخص'!$C$10</f>
+        <v>1118.5</v>
+      </c>
+      <c r="F7" s="19">
+        <f>E7+D7</f>
+        <v>1119.1</v>
+      </c>
+      <c r="G7" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H8</f>
+        <v>169.21500000000532</v>
+      </c>
+      <c r="H7" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J8</f>
+        <v>29.175</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="J7" s="19">
+        <f>I7*D7</f>
+        <v>20.424</v>
+      </c>
+      <c r="K7" s="37" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="L7" s="19">
+        <f>'الملخص'!$C$7-F7</f>
+        <v>1.800000000000182</v>
+      </c>
+      <c r="M7" s="19">
+        <f>K7*L7</f>
+        <v>14.976000000001514</v>
+      </c>
+      <c r="N7" s="38">
+        <f>G7-H7-J7-M7</f>
+        <v>104.64000000000378</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P1</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E8" s="14">
+        <f>'الملخص'!$C$10</f>
+        <v>1118.5</v>
+      </c>
+      <c r="F8" s="35">
+        <f>E8+D8</f>
+        <v>1119.1</v>
+      </c>
+      <c r="G8" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H9</f>
+        <v>82.15700000000257</v>
+      </c>
+      <c r="H8" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J9</f>
+        <v>14.165</v>
+      </c>
+      <c r="I8" s="34" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="J8" s="35">
+        <f>I8*D8</f>
+        <v>7.776</v>
+      </c>
+      <c r="K8" s="34" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="L8" s="35">
+        <f>'الملخص'!$C$7-F8</f>
+        <v>1.800000000000182</v>
+      </c>
+      <c r="M8" s="35">
+        <f>K8*L8</f>
+        <v>0.8820000000000892</v>
+      </c>
+      <c r="N8" s="36">
+        <f>G8-H8-J8-M8</f>
+        <v>59.33400000000249</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P2</t>
+        </is>
+      </c>
+      <c r="D9" s="37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="15">
+        <f>'الملخص'!$C$10</f>
+        <v>1118.5</v>
+      </c>
+      <c r="F9" s="19">
+        <f>E9+D9</f>
+        <v>1119.0</v>
+      </c>
+      <c r="G9" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H10</f>
+        <v>47.24100000000148</v>
+      </c>
+      <c r="H9" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J10</f>
+        <v>8.145</v>
+      </c>
+      <c r="I9" s="37" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="J9" s="19">
+        <f>I9*D9</f>
+        <v>2.185</v>
+      </c>
+      <c r="K9" s="37" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="L9" s="19">
+        <f>'الملخص'!$C$7-F9</f>
+        <v>1.900000000000091</v>
+      </c>
+      <c r="M9" s="19">
+        <f>K9*L9</f>
+        <v>0.6080000000000291</v>
+      </c>
+      <c r="N9" s="38">
+        <f>G9-H9-J9-M9</f>
+        <v>36.30300000000145</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P3</t>
+        </is>
+      </c>
+      <c r="D10" s="34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="14">
+        <f>'الملخص'!$C$10</f>
+        <v>1118.5</v>
+      </c>
+      <c r="F10" s="35">
+        <f>E10+D10</f>
+        <v>1119.0</v>
+      </c>
+      <c r="G10" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!H11</f>
+        <v>37.323000000001166</v>
+      </c>
+      <c r="H10" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!J11</f>
+        <v>6.435</v>
+      </c>
+      <c r="I10" s="34" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="J10" s="35">
+        <f>I10*D10</f>
+        <v>2.185</v>
+      </c>
+      <c r="K10" s="34" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="L10" s="35">
+        <f>'الملخص'!$C$7-F10</f>
+        <v>1.900000000000091</v>
+      </c>
+      <c r="M10" s="35">
+        <f>K10*L10</f>
+        <v>0.6080000000000291</v>
+      </c>
+      <c r="N10" s="36">
+        <f>G10-H10-J10-M10</f>
+        <v>28.09500000000114</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="n"/>
+      <c r="D11" s="41" t="n"/>
+      <c r="E11" s="41" t="n"/>
+      <c r="F11" s="41" t="n"/>
+      <c r="G11" s="41">
+        <f>SUM(G6:G10)</f>
+        <v>1072.5360000000337</v>
+      </c>
+      <c r="H11" s="41">
+        <f>SUM(H6:H10)</f>
+        <v>184.92000000000002</v>
+      </c>
+      <c r="I11" s="41">
+        <f>SUM(I6:I10)</f>
+        <v>221.35000000000002</v>
+      </c>
+      <c r="J11" s="41">
+        <f>SUM(J6:J10)</f>
+        <v>131.93599999999998</v>
+      </c>
+      <c r="K11" s="41">
+        <f>SUM(K6:K10)</f>
+        <v>38.50000000000001</v>
+      </c>
+      <c r="L11" s="41" t="n"/>
+      <c r="M11" s="41">
+        <f>SUM(M6:M10)</f>
+        <v>69.36400000000695</v>
+      </c>
+      <c r="N11" s="41">
+        <f>SUM(N6:N10)</f>
+        <v>686.3160000000266</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>ثانياً: قبل – القواعد على منسوب 1118.0 مباشرة، الحفر على مساحة النظافة</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>القاعدة</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>سماكة القاعدة
+(م)</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>منسوب أسفل
+القاعدة</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>منسوب سطح
+القاعدة</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>الحفر
 (م³)</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="41" t="inlineStr"/>
-      <c r="C6" s="41" t="inlineStr"/>
-      <c r="D6" s="41" t="inlineStr">
-        <is>
-          <t>من الرسم</t>
-        </is>
-      </c>
-      <c r="E6" s="41" t="inlineStr">
-        <is>
-          <t>من الرسم</t>
-        </is>
-      </c>
-      <c r="F6" s="41" t="inlineStr">
-        <is>
-          <t>سيكلوبين − نظافة</t>
-        </is>
-      </c>
-      <c r="G6" s="41" t="inlineStr">
-        <is>
-          <t>نظافة × عمق الحفر</t>
-        </is>
-      </c>
-      <c r="H6" s="41" t="inlineStr">
-        <is>
-          <t>سيكلوبين × عمق الحفر</t>
-        </is>
-      </c>
-      <c r="I6" s="41" t="inlineStr">
-        <is>
-          <t>بعد − قبل</t>
-        </is>
-      </c>
-      <c r="J6" s="41" t="inlineStr">
-        <is>
-          <t>سيكلوبين × السماكة</t>
-        </is>
-      </c>
-      <c r="K6" s="41" t="inlineStr">
-        <is>
-          <t>شريط × ارتفاع الردم</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="7" t="n">
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>السيكلوبين
+(م³)</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>مساحة خرسانة
+القاعدة (م²)</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>خرسانة القاعدة
+(م³)</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>مساحة الرقاب
+والجدران (م²)</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>ارتفاع الرقاب
+(م)</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>حجم الرقاب
+والجدران (م³)</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>الردم
+(م³)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>قاعدة الجدار الاستنادي – الجزء الشمالي والشرقي</t>
         </is>
       </c>
-      <c r="D7" s="42" t="n">
-        <v>180.09</v>
-      </c>
-      <c r="E7" s="42" t="n">
-        <v>254</v>
-      </c>
-      <c r="F7" s="27">
-        <f>E7-D7</f>
-        <v>73.91</v>
-      </c>
-      <c r="G7" s="27">
-        <f>D7*'الملخص'!$C$11</f>
+      <c r="D15" s="34" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E15" s="14">
+        <f>'الملخص'!$C$8</f>
+        <v>1118.0</v>
+      </c>
+      <c r="F15" s="35">
+        <f>E15+D15</f>
+        <v>1118.6</v>
+      </c>
+      <c r="G15" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G7</f>
         <v>522.2610000000163</v>
       </c>
-      <c r="H7" s="27">
-        <f>E7*'الملخص'!$C$11</f>
-        <v>736.6000000000231</v>
-      </c>
-      <c r="I7" s="43">
-        <f>H7-G7</f>
-        <v>214.33900000000676</v>
-      </c>
-      <c r="J7" s="43">
-        <f>E7*'الملخص'!$C$9</f>
-        <v>127.0</v>
-      </c>
-      <c r="K7" s="43">
-        <f>F7*'الملخص'!$C$12</f>
-        <v>177.38400000000672</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="10" t="n">
+      <c r="H15" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="34" t="n">
+        <v>165.61</v>
+      </c>
+      <c r="J15" s="35">
+        <f>I15*D15</f>
+        <v>99.366</v>
+      </c>
+      <c r="K15" s="34" t="n">
+        <v>29.05</v>
+      </c>
+      <c r="L15" s="35">
+        <f>'الملخص'!$C$7-F15</f>
+        <v>2.300000000000182</v>
+      </c>
+      <c r="M15" s="35">
+        <f>K15*L15</f>
+        <v>66.81500000000528</v>
+      </c>
+      <c r="N15" s="36">
+        <f>G15-H15-J15-M15</f>
+        <v>356.08000000001107</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>قاعدة الجدار الاستنادي – الجزء الجنوبي والمنحنى</t>
         </is>
       </c>
-      <c r="D8" s="44" t="n">
-        <v>38.65</v>
-      </c>
-      <c r="E8" s="44" t="n">
-        <v>58.35</v>
-      </c>
-      <c r="F8" s="31">
-        <f>E8-D8</f>
-        <v>19.700000000000003</v>
-      </c>
-      <c r="G8" s="31">
-        <f>D8*'الملخص'!$C$11</f>
+      <c r="D16" s="37" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E16" s="15">
+        <f>'الملخص'!$C$8</f>
+        <v>1118.0</v>
+      </c>
+      <c r="F16" s="19">
+        <f>E16+D16</f>
+        <v>1118.6</v>
+      </c>
+      <c r="G16" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G8</f>
         <v>112.08500000000352</v>
       </c>
-      <c r="H8" s="31">
-        <f>E8*'الملخص'!$C$11</f>
-        <v>169.21500000000532</v>
-      </c>
-      <c r="I8" s="45">
-        <f>H8-G8</f>
-        <v>57.1300000000018</v>
-      </c>
-      <c r="J8" s="45">
-        <f>E8*'الملخص'!$C$9</f>
-        <v>29.175</v>
-      </c>
-      <c r="K8" s="45">
-        <f>F8*'الملخص'!$C$12</f>
-        <v>47.2800000000018</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="7" t="n">
+      <c r="H16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="37" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="J16" s="19">
+        <f>I16*D16</f>
+        <v>20.424</v>
+      </c>
+      <c r="K16" s="37" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="L16" s="19">
+        <f>'الملخص'!$C$7-F16</f>
+        <v>2.300000000000182</v>
+      </c>
+      <c r="M16" s="19">
+        <f>K16*L16</f>
+        <v>19.136000000001513</v>
+      </c>
+      <c r="N16" s="38">
+        <f>G16-H16-J16-M16</f>
+        <v>72.52500000000201</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>قاعدة منفصلة P1</t>
         </is>
       </c>
-      <c r="D9" s="42" t="n">
-        <v>14.44</v>
-      </c>
-      <c r="E9" s="42" t="n">
-        <v>28.33</v>
-      </c>
-      <c r="F9" s="27">
-        <f>E9-D9</f>
-        <v>13.889999999999999</v>
-      </c>
-      <c r="G9" s="27">
-        <f>D9*'الملخص'!$C$11</f>
+      <c r="D17" s="34" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E17" s="14">
+        <f>'الملخص'!$C$8</f>
+        <v>1118.0</v>
+      </c>
+      <c r="F17" s="35">
+        <f>E17+D17</f>
+        <v>1118.6</v>
+      </c>
+      <c r="G17" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G9</f>
         <v>41.87600000000131</v>
       </c>
-      <c r="H9" s="27">
-        <f>E9*'الملخص'!$C$11</f>
-        <v>82.15700000000257</v>
-      </c>
-      <c r="I9" s="43">
-        <f>H9-G9</f>
-        <v>40.28100000000126</v>
-      </c>
-      <c r="J9" s="43">
-        <f>E9*'الملخص'!$C$9</f>
-        <v>14.165</v>
-      </c>
-      <c r="K9" s="43">
-        <f>F9*'الملخص'!$C$12</f>
-        <v>33.33600000000126</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="10" t="n">
+      <c r="H17" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="34" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="J17" s="35">
+        <f>I17*D17</f>
+        <v>7.776</v>
+      </c>
+      <c r="K17" s="34" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="L17" s="35">
+        <f>'الملخص'!$C$7-F17</f>
+        <v>2.300000000000182</v>
+      </c>
+      <c r="M17" s="35">
+        <f>K17*L17</f>
+        <v>1.127000000000089</v>
+      </c>
+      <c r="N17" s="36">
+        <f>G17-H17-J17-M17</f>
+        <v>32.97300000000123</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>قاعدة منفصلة P2</t>
         </is>
       </c>
-      <c r="D10" s="44" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="E10" s="44" t="n">
-        <v>16.29</v>
-      </c>
-      <c r="F10" s="31">
-        <f>E10-D10</f>
-        <v>11.04</v>
-      </c>
-      <c r="G10" s="31">
-        <f>D10*'الملخص'!$C$11</f>
+      <c r="D18" s="37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E18" s="15">
+        <f>'الملخص'!$C$8</f>
+        <v>1118.0</v>
+      </c>
+      <c r="F18" s="19">
+        <f>E18+D18</f>
+        <v>1118.5</v>
+      </c>
+      <c r="G18" s="15">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G10</f>
         <v>15.225000000000477</v>
       </c>
-      <c r="H10" s="31">
-        <f>E10*'الملخص'!$C$11</f>
-        <v>47.24100000000148</v>
-      </c>
-      <c r="I10" s="45">
-        <f>H10-G10</f>
-        <v>32.016000000001</v>
-      </c>
-      <c r="J10" s="45">
-        <f>E10*'الملخص'!$C$9</f>
-        <v>8.145</v>
-      </c>
-      <c r="K10" s="45">
-        <f>F10*'الملخص'!$C$12</f>
-        <v>26.496000000001</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="7" t="n">
+      <c r="H18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="37" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="J18" s="19">
+        <f>I18*D18</f>
+        <v>2.185</v>
+      </c>
+      <c r="K18" s="37" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="L18" s="19">
+        <f>'الملخص'!$C$7-F18</f>
+        <v>2.400000000000091</v>
+      </c>
+      <c r="M18" s="19">
+        <f>K18*L18</f>
+        <v>0.7680000000000291</v>
+      </c>
+      <c r="N18" s="38">
+        <f>G18-H18-J18-M18</f>
+        <v>12.272000000000448</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>قاعدة منفصلة P3</t>
         </is>
       </c>
-      <c r="D11" s="42" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="E11" s="42" t="n">
-        <v>12.87</v>
-      </c>
-      <c r="F11" s="27">
-        <f>E11-D11</f>
-        <v>7.619999999999999</v>
-      </c>
-      <c r="G11" s="27">
-        <f>D11*'الملخص'!$C$11</f>
+      <c r="D19" s="34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E19" s="14">
+        <f>'الملخص'!$C$8</f>
+        <v>1118.0</v>
+      </c>
+      <c r="F19" s="35">
+        <f>E19+D19</f>
+        <v>1118.5</v>
+      </c>
+      <c r="G19" s="14">
+        <f>'الإزاحة 1 م من وجه الخرسانة'!G11</f>
         <v>15.225000000000477</v>
       </c>
-      <c r="H11" s="27">
-        <f>E11*'الملخص'!$C$11</f>
-        <v>37.323000000001166</v>
-      </c>
-      <c r="I11" s="43">
-        <f>H11-G11</f>
-        <v>22.098000000000688</v>
-      </c>
-      <c r="J11" s="43">
-        <f>E11*'الملخص'!$C$9</f>
-        <v>6.435</v>
-      </c>
-      <c r="K11" s="43">
-        <f>F11*'الملخص'!$C$12</f>
-        <v>18.28800000000069</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="33" t="inlineStr">
+      <c r="H19" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="34" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="J19" s="35">
+        <f>I19*D19</f>
+        <v>2.185</v>
+      </c>
+      <c r="K19" s="34" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="L19" s="35">
+        <f>'الملخص'!$C$7-F19</f>
+        <v>2.400000000000091</v>
+      </c>
+      <c r="M19" s="35">
+        <f>K19*L19</f>
+        <v>0.7680000000000291</v>
+      </c>
+      <c r="N19" s="36">
+        <f>G19-H19-J19-M19</f>
+        <v>12.272000000000448</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="39" t="inlineStr">
         <is>
           <t>المجموع</t>
         </is>
       </c>
-      <c r="C12" s="34" t="n"/>
-      <c r="D12" s="38">
-        <f>SUM(D7:D11)</f>
-        <v>243.68</v>
-      </c>
-      <c r="E12" s="38">
-        <f>SUM(E7:E11)</f>
-        <v>369.84000000000003</v>
-      </c>
-      <c r="F12" s="38">
-        <f>SUM(F7:F11)</f>
-        <v>126.16</v>
-      </c>
-      <c r="G12" s="38">
-        <f>SUM(G7:G11)</f>
+      <c r="C20" s="40" t="n"/>
+      <c r="D20" s="41" t="n"/>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="41">
+        <f>SUM(G15:G19)</f>
         <v>706.6720000000222</v>
       </c>
-      <c r="H12" s="38">
-        <f>SUM(H7:H11)</f>
-        <v>1072.5360000000337</v>
-      </c>
-      <c r="I12" s="38">
-        <f>SUM(I7:I11)</f>
-        <v>365.8640000000115</v>
-      </c>
-      <c r="J12" s="38">
-        <f>SUM(J7:J11)</f>
-        <v>184.92000000000002</v>
-      </c>
-      <c r="K12" s="38">
-        <f>SUM(K7:K11)</f>
-        <v>302.7840000000115</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="39" t="inlineStr">
+      <c r="H20" s="41">
+        <f>SUM(H15:H19)</f>
+        <v>0.0</v>
+      </c>
+      <c r="I20" s="41">
+        <f>SUM(I15:I19)</f>
+        <v>221.35000000000002</v>
+      </c>
+      <c r="J20" s="41">
+        <f>SUM(J15:J19)</f>
+        <v>131.93599999999998</v>
+      </c>
+      <c r="K20" s="41">
+        <f>SUM(K15:K19)</f>
+        <v>38.50000000000001</v>
+      </c>
+      <c r="L20" s="41" t="n"/>
+      <c r="M20" s="41">
+        <f>SUM(M15:M19)</f>
+        <v>88.61400000000695</v>
+      </c>
+      <c r="N20" s="41">
+        <f>SUM(N15:N19)</f>
+        <v>486.1220000000152</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>ملاحظات:</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="40" t="inlineStr">
-        <is>
-          <t>• مساحات النظافة والسيكلوبين مقيسة من ملف syclopien.dxf (التهشير الرمادي على طبقة S-D-WATER PROOF، وهو مرسوم على حد النظافة).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t>• في أماكن تداخل إزاحات القواعد المتجاورة وُزّعت المساحة المشتركة على أقرب قاعدة حتى لا تُحسب مرتين.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="40" t="inlineStr">
-        <is>
-          <t>• الحفر الزائد = توسيع حفر القواعد بشريط الإزاحة من المنسوب العام حتى منسوب الحفر النهائي؛ لا يوجد حفر تحت هذا المنسوب.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="40" t="inlineStr">
-        <is>
-          <t>• الردم الزائد = شريط الإزاحة فوق السيكلوبين حتى المنسوب العام. لا يشمل الردم فوق القواعد نفسها لأنه موجود في الحالتين.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="40" t="inlineStr">
-        <is>
-          <t>• الجوانب محسوبة رأسية؛ أي ميول في جوانب الحفر تزيد الحفر والردم.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="40" t="inlineStr">
-        <is>
-          <t>• الخلايا الزرقاء قيم مقيسة من الرسم، والباقي معادلات مرتبطة بصفحة الملخص.</t>
+    <row r="23">
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>• سماكات القواعد: قاعدة الجدار الاستنادي 60 سم (RAFT Thickness 60cm في الرسم)، F3 = 60 سم، F2 = 50 سم (جدول القواعد).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>• مساحة خرسانة القاعدة = خط التهشير مُزاحاً 10 سم للداخل (التهشير مرسوم على حد النظافة).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>• الرقاب والجدران: الأعمدة (S-S-COLUMN HATCH) والجدار الاستنادي والجدران الواقعة فوق القواعد، من سطح القاعدة حتى 1120.9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>• لم تُخصم الجسور الأرضية (G.B1) ولا خرسانة النظافة في حالة "قبل" – تحتاج مقاطعها وسماكتها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>• الخلايا الزرقاء من الرسم أو جدول القواعد، والخضراء مرتبطة بصفحات أخرى، والباقي معادلات.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B14:K14"/>
-    <mergeCell ref="B17:K17"/>
-    <mergeCell ref="B18:K18"/>
-    <mergeCell ref="B16:K16"/>
-    <mergeCell ref="B15:K15"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B20:K20"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B19:K19"/>
-    <mergeCell ref="B12:C12"/>
+  <mergeCells count="12">
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B22:N22"/>
+    <mergeCell ref="B23:N23"/>
+    <mergeCell ref="B3:M3"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B27:N27"/>
+    <mergeCell ref="B4:N4"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B26:N26"/>
+    <mergeCell ref="B13:N13"/>
+    <mergeCell ref="B25:N25"/>
+    <mergeCell ref="B24:N24"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2099,14 +2570,14 @@
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>جدول تفصيلي – بديل - الإزاحة من حد النظافة</t>
+          <t>جدول تفصيلي – الإزاحة 1 م من وجه الخرسانة</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>للمقارنة فقط: الإزاحة 1.0 م مقيسة من خط التهشير (حد النظافة) – بدون إزاحة على الوجه الخارجي للجدار الاستنادي</t>
+          <t>المعتمد: الإزاحة 1.0 م مقيسة من وجه الخرسانة (0.9 م من حد النظافة) – بدون إزاحة على الوجه الخارجي للجدار الاستنادي</t>
         </is>
       </c>
     </row>
@@ -2167,50 +2638,50 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>الردم الزائد
-(م³)</t>
+          <t>ردم شريط الإزاحة
+فوق السيكلوبين (م³)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="41" t="inlineStr"/>
-      <c r="C6" s="41" t="inlineStr"/>
-      <c r="D6" s="41" t="inlineStr">
+      <c r="B6" s="42" t="inlineStr"/>
+      <c r="C6" s="42" t="inlineStr"/>
+      <c r="D6" s="42" t="inlineStr">
         <is>
           <t>من الرسم</t>
         </is>
       </c>
-      <c r="E6" s="41" t="inlineStr">
+      <c r="E6" s="42" t="inlineStr">
         <is>
           <t>من الرسم</t>
         </is>
       </c>
-      <c r="F6" s="41" t="inlineStr">
+      <c r="F6" s="42" t="inlineStr">
         <is>
           <t>سيكلوبين − نظافة</t>
         </is>
       </c>
-      <c r="G6" s="41" t="inlineStr">
+      <c r="G6" s="42" t="inlineStr">
         <is>
           <t>نظافة × عمق الحفر</t>
         </is>
       </c>
-      <c r="H6" s="41" t="inlineStr">
+      <c r="H6" s="42" t="inlineStr">
         <is>
           <t>سيكلوبين × عمق الحفر</t>
         </is>
       </c>
-      <c r="I6" s="41" t="inlineStr">
+      <c r="I6" s="42" t="inlineStr">
         <is>
           <t>بعد − قبل</t>
         </is>
       </c>
-      <c r="J6" s="41" t="inlineStr">
+      <c r="J6" s="42" t="inlineStr">
         <is>
           <t>سيكلوبين × السماكة</t>
         </is>
       </c>
-      <c r="K6" s="41" t="inlineStr">
+      <c r="K6" s="42" t="inlineStr">
         <is>
           <t>شريط × ارتفاع الردم</t>
         </is>
@@ -2225,35 +2696,35 @@
           <t>قاعدة الجدار الاستنادي – الجزء الشمالي والشرقي</t>
         </is>
       </c>
-      <c r="D7" s="42" t="n">
+      <c r="D7" s="34" t="n">
         <v>180.09</v>
       </c>
-      <c r="E7" s="42" t="n">
-        <v>262.24</v>
-      </c>
-      <c r="F7" s="27">
+      <c r="E7" s="34" t="n">
+        <v>254</v>
+      </c>
+      <c r="F7" s="35">
         <f>E7-D7</f>
-        <v>82.15</v>
-      </c>
-      <c r="G7" s="27">
+        <v>73.91</v>
+      </c>
+      <c r="G7" s="35">
         <f>D7*'الملخص'!$C$11</f>
         <v>522.2610000000163</v>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="35">
         <f>E7*'الملخص'!$C$11</f>
-        <v>760.4960000000239</v>
-      </c>
-      <c r="I7" s="43">
+        <v>736.6000000000231</v>
+      </c>
+      <c r="I7" s="36">
         <f>H7-G7</f>
-        <v>238.23500000000752</v>
-      </c>
-      <c r="J7" s="43">
+        <v>214.33900000000676</v>
+      </c>
+      <c r="J7" s="36">
         <f>E7*'الملخص'!$C$9</f>
-        <v>131.12</v>
-      </c>
-      <c r="K7" s="43">
+        <v>127.0</v>
+      </c>
+      <c r="K7" s="36">
         <f>F7*'الملخص'!$C$12</f>
-        <v>197.16000000000747</v>
+        <v>177.38400000000672</v>
       </c>
     </row>
     <row r="8">
@@ -2265,35 +2736,35 @@
           <t>قاعدة الجدار الاستنادي – الجزء الجنوبي والمنحنى</t>
         </is>
       </c>
-      <c r="D8" s="44" t="n">
+      <c r="D8" s="37" t="n">
         <v>38.65</v>
       </c>
-      <c r="E8" s="44" t="n">
-        <v>60.51</v>
-      </c>
-      <c r="F8" s="31">
+      <c r="E8" s="37" t="n">
+        <v>58.35</v>
+      </c>
+      <c r="F8" s="19">
         <f>E8-D8</f>
-        <v>21.86</v>
-      </c>
-      <c r="G8" s="31">
+        <v>19.700000000000003</v>
+      </c>
+      <c r="G8" s="19">
         <f>D8*'الملخص'!$C$11</f>
         <v>112.08500000000352</v>
       </c>
-      <c r="H8" s="31">
+      <c r="H8" s="19">
         <f>E8*'الملخص'!$C$11</f>
-        <v>175.4790000000055</v>
-      </c>
-      <c r="I8" s="45">
+        <v>169.21500000000532</v>
+      </c>
+      <c r="I8" s="38">
         <f>H8-G8</f>
-        <v>63.39400000000198</v>
-      </c>
-      <c r="J8" s="45">
+        <v>57.1300000000018</v>
+      </c>
+      <c r="J8" s="38">
         <f>E8*'الملخص'!$C$9</f>
-        <v>30.255</v>
-      </c>
-      <c r="K8" s="45">
+        <v>29.175</v>
+      </c>
+      <c r="K8" s="38">
         <f>F8*'الملخص'!$C$12</f>
-        <v>52.46400000000199</v>
+        <v>47.2800000000018</v>
       </c>
     </row>
     <row r="9">
@@ -2305,35 +2776,35 @@
           <t>قاعدة منفصلة P1</t>
         </is>
       </c>
-      <c r="D9" s="42" t="n">
+      <c r="D9" s="34" t="n">
         <v>14.44</v>
       </c>
-      <c r="E9" s="42" t="n">
-        <v>29.95</v>
-      </c>
-      <c r="F9" s="27">
+      <c r="E9" s="34" t="n">
+        <v>28.33</v>
+      </c>
+      <c r="F9" s="35">
         <f>E9-D9</f>
-        <v>15.51</v>
-      </c>
-      <c r="G9" s="27">
+        <v>13.889999999999999</v>
+      </c>
+      <c r="G9" s="35">
         <f>D9*'الملخص'!$C$11</f>
         <v>41.87600000000131</v>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="35">
         <f>E9*'الملخص'!$C$11</f>
-        <v>86.85500000000272</v>
-      </c>
-      <c r="I9" s="43">
+        <v>82.15700000000257</v>
+      </c>
+      <c r="I9" s="36">
         <f>H9-G9</f>
-        <v>44.979000000001406</v>
-      </c>
-      <c r="J9" s="43">
+        <v>40.28100000000126</v>
+      </c>
+      <c r="J9" s="36">
         <f>E9*'الملخص'!$C$9</f>
-        <v>14.975</v>
-      </c>
-      <c r="K9" s="43">
+        <v>14.165</v>
+      </c>
+      <c r="K9" s="36">
         <f>F9*'الملخص'!$C$12</f>
-        <v>37.22400000000141</v>
+        <v>33.33600000000126</v>
       </c>
     </row>
     <row r="10">
@@ -2345,35 +2816,35 @@
           <t>قاعدة منفصلة P2</t>
         </is>
       </c>
-      <c r="D10" s="44" t="n">
+      <c r="D10" s="37" t="n">
         <v>5.25</v>
       </c>
-      <c r="E10" s="44" t="n">
-        <v>17.73</v>
-      </c>
-      <c r="F10" s="31">
+      <c r="E10" s="37" t="n">
+        <v>16.29</v>
+      </c>
+      <c r="F10" s="19">
         <f>E10-D10</f>
-        <v>12.48</v>
-      </c>
-      <c r="G10" s="31">
+        <v>11.04</v>
+      </c>
+      <c r="G10" s="19">
         <f>D10*'الملخص'!$C$11</f>
         <v>15.225000000000477</v>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="19">
         <f>E10*'الملخص'!$C$11</f>
-        <v>51.417000000001615</v>
-      </c>
-      <c r="I10" s="45">
+        <v>47.24100000000148</v>
+      </c>
+      <c r="I10" s="38">
         <f>H10-G10</f>
-        <v>36.19200000000114</v>
-      </c>
-      <c r="J10" s="45">
+        <v>32.016000000001</v>
+      </c>
+      <c r="J10" s="38">
         <f>E10*'الملخص'!$C$9</f>
-        <v>8.865</v>
-      </c>
-      <c r="K10" s="45">
+        <v>8.145</v>
+      </c>
+      <c r="K10" s="38">
         <f>F10*'الملخص'!$C$12</f>
-        <v>29.952000000001135</v>
+        <v>26.496000000001</v>
       </c>
     </row>
     <row r="11">
@@ -2385,121 +2856,572 @@
           <t>قاعدة منفصلة P3</t>
         </is>
       </c>
-      <c r="D11" s="42" t="n">
+      <c r="D11" s="34" t="n">
         <v>5.25</v>
       </c>
-      <c r="E11" s="42" t="n">
+      <c r="E11" s="34" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="F11" s="35">
+        <f>E11-D11</f>
+        <v>7.619999999999999</v>
+      </c>
+      <c r="G11" s="35">
+        <f>D11*'الملخص'!$C$11</f>
+        <v>15.225000000000477</v>
+      </c>
+      <c r="H11" s="35">
+        <f>E11*'الملخص'!$C$11</f>
+        <v>37.323000000001166</v>
+      </c>
+      <c r="I11" s="36">
+        <f>H11-G11</f>
+        <v>22.098000000000688</v>
+      </c>
+      <c r="J11" s="36">
+        <f>E11*'الملخص'!$C$9</f>
+        <v>6.435</v>
+      </c>
+      <c r="K11" s="36">
+        <f>F11*'الملخص'!$C$12</f>
+        <v>18.28800000000069</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="41">
+        <f>SUM(D7:D11)</f>
+        <v>243.68</v>
+      </c>
+      <c r="E12" s="41">
+        <f>SUM(E7:E11)</f>
+        <v>369.84000000000003</v>
+      </c>
+      <c r="F12" s="41">
+        <f>SUM(F7:F11)</f>
+        <v>126.16</v>
+      </c>
+      <c r="G12" s="41">
+        <f>SUM(G7:G11)</f>
+        <v>706.6720000000222</v>
+      </c>
+      <c r="H12" s="41">
+        <f>SUM(H7:H11)</f>
+        <v>1072.5360000000337</v>
+      </c>
+      <c r="I12" s="41">
+        <f>SUM(I7:I11)</f>
+        <v>365.8640000000115</v>
+      </c>
+      <c r="J12" s="41">
+        <f>SUM(J7:J11)</f>
+        <v>184.92000000000002</v>
+      </c>
+      <c r="K12" s="41">
+        <f>SUM(K7:K11)</f>
+        <v>302.7840000000115</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>ملاحظات:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>• مساحات النظافة والسيكلوبين مقيسة من ملف syclopien.dxf (التهشير الرمادي على طبقة S-D-WATER PROOF، وهو مرسوم على حد النظافة).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>• في أماكن تداخل إزاحات القواعد المتجاورة وُزّعت المساحة المشتركة على أقرب قاعدة حتى لا تُحسب مرتين.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>• الحفر الزائد = توسيع حفر القواعد بشريط الإزاحة من المنسوب العام حتى منسوب الحفر النهائي؛ لا يوجد حفر تحت هذا المنسوب.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>• الردم الزائد = شريط الإزاحة فوق السيكلوبين حتى المنسوب العام. لا يشمل الردم فوق القواعد نفسها لأنه موجود في الحالتين.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>• الجوانب محسوبة رأسية؛ أي ميول في جوانب الحفر تزيد الحفر والردم.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>• الخلايا الزرقاء قيم مقيسة من الرسم، والباقي معادلات مرتبطة بصفحة الملخص.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B14:K14"/>
+    <mergeCell ref="B17:K17"/>
+    <mergeCell ref="B18:K18"/>
+    <mergeCell ref="B16:K16"/>
+    <mergeCell ref="B15:K15"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B20:K20"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B19:K19"/>
+    <mergeCell ref="B12:C12"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:K20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="2" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>جدول تفصيلي – بديل - الإزاحة من حد النظافة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>للمقارنة فقط: الإزاحة 1.0 م مقيسة من خط التهشير (حد النظافة) – بدون إزاحة على الوجه الخارجي للجدار الاستنادي</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>القاعدة</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>مساحة النظافة
+(م²)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>مساحة السيكلوبين
+(م²)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>مساحة شريط الإزاحة
+(م²)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>الحفر قبل
+على مساحة النظافة
+(م³)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>الحفر بعد
+على مساحة السيكلوبين
+(م³)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>الحفر الزائد
+(م³)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>خرسانة السيكلوبين
+(م³)</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>ردم شريط الإزاحة
+فوق السيكلوبين (م³)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="42" t="inlineStr"/>
+      <c r="C6" s="42" t="inlineStr"/>
+      <c r="D6" s="42" t="inlineStr">
+        <is>
+          <t>من الرسم</t>
+        </is>
+      </c>
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>من الرسم</t>
+        </is>
+      </c>
+      <c r="F6" s="42" t="inlineStr">
+        <is>
+          <t>سيكلوبين − نظافة</t>
+        </is>
+      </c>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>نظافة × عمق الحفر</t>
+        </is>
+      </c>
+      <c r="H6" s="42" t="inlineStr">
+        <is>
+          <t>سيكلوبين × عمق الحفر</t>
+        </is>
+      </c>
+      <c r="I6" s="42" t="inlineStr">
+        <is>
+          <t>بعد − قبل</t>
+        </is>
+      </c>
+      <c r="J6" s="42" t="inlineStr">
+        <is>
+          <t>سيكلوبين × السماكة</t>
+        </is>
+      </c>
+      <c r="K6" s="42" t="inlineStr">
+        <is>
+          <t>شريط × ارتفاع الردم</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة الجدار الاستنادي – الجزء الشمالي والشرقي</t>
+        </is>
+      </c>
+      <c r="D7" s="34" t="n">
+        <v>180.09</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>262.24</v>
+      </c>
+      <c r="F7" s="35">
+        <f>E7-D7</f>
+        <v>82.15</v>
+      </c>
+      <c r="G7" s="35">
+        <f>D7*'الملخص'!$C$11</f>
+        <v>522.2610000000163</v>
+      </c>
+      <c r="H7" s="35">
+        <f>E7*'الملخص'!$C$11</f>
+        <v>760.4960000000239</v>
+      </c>
+      <c r="I7" s="36">
+        <f>H7-G7</f>
+        <v>238.23500000000752</v>
+      </c>
+      <c r="J7" s="36">
+        <f>E7*'الملخص'!$C$9</f>
+        <v>131.12</v>
+      </c>
+      <c r="K7" s="36">
+        <f>F7*'الملخص'!$C$12</f>
+        <v>197.16000000000747</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>قاعدة الجدار الاستنادي – الجزء الجنوبي والمنحنى</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="E8" s="37" t="n">
+        <v>60.51</v>
+      </c>
+      <c r="F8" s="19">
+        <f>E8-D8</f>
+        <v>21.86</v>
+      </c>
+      <c r="G8" s="19">
+        <f>D8*'الملخص'!$C$11</f>
+        <v>112.08500000000352</v>
+      </c>
+      <c r="H8" s="19">
+        <f>E8*'الملخص'!$C$11</f>
+        <v>175.4790000000055</v>
+      </c>
+      <c r="I8" s="38">
+        <f>H8-G8</f>
+        <v>63.39400000000198</v>
+      </c>
+      <c r="J8" s="38">
+        <f>E8*'الملخص'!$C$9</f>
+        <v>30.255</v>
+      </c>
+      <c r="K8" s="38">
+        <f>F8*'الملخص'!$C$12</f>
+        <v>52.46400000000199</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P1</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>14.44</v>
+      </c>
+      <c r="E9" s="34" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="F9" s="35">
+        <f>E9-D9</f>
+        <v>15.51</v>
+      </c>
+      <c r="G9" s="35">
+        <f>D9*'الملخص'!$C$11</f>
+        <v>41.87600000000131</v>
+      </c>
+      <c r="H9" s="35">
+        <f>E9*'الملخص'!$C$11</f>
+        <v>86.85500000000272</v>
+      </c>
+      <c r="I9" s="36">
+        <f>H9-G9</f>
+        <v>44.979000000001406</v>
+      </c>
+      <c r="J9" s="36">
+        <f>E9*'الملخص'!$C$9</f>
+        <v>14.975</v>
+      </c>
+      <c r="K9" s="36">
+        <f>F9*'الملخص'!$C$12</f>
+        <v>37.22400000000141</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P2</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="E10" s="37" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="F10" s="19">
+        <f>E10-D10</f>
+        <v>12.48</v>
+      </c>
+      <c r="G10" s="19">
+        <f>D10*'الملخص'!$C$11</f>
+        <v>15.225000000000477</v>
+      </c>
+      <c r="H10" s="19">
+        <f>E10*'الملخص'!$C$11</f>
+        <v>51.417000000001615</v>
+      </c>
+      <c r="I10" s="38">
+        <f>H10-G10</f>
+        <v>36.19200000000114</v>
+      </c>
+      <c r="J10" s="38">
+        <f>E10*'الملخص'!$C$9</f>
+        <v>8.865</v>
+      </c>
+      <c r="K10" s="38">
+        <f>F10*'الملخص'!$C$12</f>
+        <v>29.952000000001135</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>قاعدة منفصلة P3</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="E11" s="34" t="n">
         <v>13.82</v>
       </c>
-      <c r="F11" s="27">
+      <c r="F11" s="35">
         <f>E11-D11</f>
         <v>8.57</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="35">
         <f>D11*'الملخص'!$C$11</f>
         <v>15.225000000000477</v>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="35">
         <f>E11*'الملخص'!$C$11</f>
         <v>40.07800000000126</v>
       </c>
-      <c r="I11" s="43">
+      <c r="I11" s="36">
         <f>H11-G11</f>
         <v>24.853000000000783</v>
       </c>
-      <c r="J11" s="43">
+      <c r="J11" s="36">
         <f>E11*'الملخص'!$C$9</f>
         <v>6.91</v>
       </c>
-      <c r="K11" s="43">
+      <c r="K11" s="36">
         <f>F11*'الملخص'!$C$12</f>
         <v>20.56800000000078</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="33" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>المجموع</t>
         </is>
       </c>
-      <c r="C12" s="34" t="n"/>
-      <c r="D12" s="38">
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="41">
         <f>SUM(D7:D11)</f>
         <v>243.68</v>
       </c>
-      <c r="E12" s="38">
+      <c r="E12" s="41">
         <f>SUM(E7:E11)</f>
         <v>384.25</v>
       </c>
-      <c r="F12" s="38">
+      <c r="F12" s="41">
         <f>SUM(F7:F11)</f>
         <v>140.57</v>
       </c>
-      <c r="G12" s="38">
+      <c r="G12" s="41">
         <f>SUM(G7:G11)</f>
         <v>706.6720000000222</v>
       </c>
-      <c r="H12" s="38">
+      <c r="H12" s="41">
         <f>SUM(H7:H11)</f>
         <v>1114.325000000035</v>
       </c>
-      <c r="I12" s="38">
+      <c r="I12" s="41">
         <f>SUM(I7:I11)</f>
         <v>407.65300000001287</v>
       </c>
-      <c r="J12" s="38">
+      <c r="J12" s="41">
         <f>SUM(J7:J11)</f>
         <v>192.125</v>
       </c>
-      <c r="K12" s="38">
+      <c r="K12" s="41">
         <f>SUM(K7:K11)</f>
         <v>337.3680000000128</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="39" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>ملاحظات:</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="40" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>• مساحات النظافة والسيكلوبين مقيسة من ملف syclopien.dxf (التهشير الرمادي على طبقة S-D-WATER PROOF، وهو مرسوم على حد النظافة).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>• في أماكن تداخل إزاحات القواعد المتجاورة وُزّعت المساحة المشتركة على أقرب قاعدة حتى لا تُحسب مرتين.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="40" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>• الحفر الزائد = توسيع حفر القواعد بشريط الإزاحة من المنسوب العام حتى منسوب الحفر النهائي؛ لا يوجد حفر تحت هذا المنسوب.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="40" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>• الردم الزائد = شريط الإزاحة فوق السيكلوبين حتى المنسوب العام. لا يشمل الردم فوق القواعد نفسها لأنه موجود في الحالتين.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="40" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>• الجوانب محسوبة رأسية؛ أي ميول في جوانب الحفر تزيد الحفر والردم.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="40" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>• الخلايا الزرقاء قيم مقيسة من الرسم، والباقي معادلات مرتبطة بصفحة الملخص.</t>
         </is>

</xml_diff>